<commit_message>
docs: change input of test case and update test case report
</commit_message>
<xml_diff>
--- a/TestCases.xlsx
+++ b/TestCases.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="89">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -40,7 +40,7 @@
     <t>TC-01</t>
   </si>
   <si>
-    <t>Verify Cool Shot Mode activation and functionality</t>
+    <t>ẻ</t>
   </si>
   <si>
     <t>Standard 220V outlet, switch at 'Cool' mode, 1 minute duration.</t>
@@ -48,10 +48,16 @@
   <si>
     <t>1. Plug the device into a standard 220V outlet.
 2. Slide the switch to the Cool mode position.
-3. Keep it running for 1 minute and feel the exhaust air.</t>
+3. Keep it running for 10s and feel the exhaust air.</t>
   </si>
   <si>
     <t>The fan rotates smoothly. The air discharged from the nozzle remains at room temperature without any heat generation.</t>
+  </si>
+  <si>
+    <t>As Expected</t>
+  </si>
+  <si>
+    <t>Pass</t>
   </si>
   <si>
     <t>TC-02</t>
@@ -84,6 +90,12 @@
   </si>
   <si>
     <t>The air speed increases noticeably compared to Position 1, and the air becomes hotter.</t>
+  </si>
+  <si>
+    <t>The air speed increased compared to Position 1, but the air temperature remained similar to Position 1.</t>
+  </si>
+  <si>
+    <t>Fail</t>
   </si>
   <si>
     <t>TC-04</t>
@@ -167,6 +179,9 @@
     <t>The loop supports the full weight of the hair dryer (approx. 400g) without tearing, excessive stretching, or letting the unit fall.</t>
   </si>
   <si>
+    <t>The hanging loop stretching after 24 hours of suspension.</t>
+  </si>
+  <si>
     <t>TC-09</t>
   </si>
   <si>
@@ -199,10 +214,13 @@
     <t>The dense honeycomb mesh safely prevents individual strands from being sucked inside the chamber or tangled into the internal fan blades.</t>
   </si>
   <si>
+    <t>Several hair strands passed through the honeycomb mesh and entered the air intake area.</t>
+  </si>
+  <si>
     <t>TC-11</t>
   </si>
   <si>
-    <t>Verify Overheating Safety Cut-off (Rơ-le tự ngắt) activation</t>
+    <t>Verify Overheating Safety Cut-off activation</t>
   </si>
   <si>
     <t>High Heat mode, solid non-flammable barrier completely blocking rear air inlet mesh.</t>
@@ -245,6 +263,9 @@
   </si>
   <si>
     <t>The handle remains cool to the touch. The barrel surface gets warm but stays safe to handle without causing minor burns or emitting burning plastic odors.</t>
+  </si>
+  <si>
+    <t>The handle became noticeably hot after 10 minutes of operation, making it uncomfortable to hold.</t>
   </si>
   <si>
     <t>TC-14</t>
@@ -283,7 +304,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -293,13 +314,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -354,11 +369,11 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -674,7 +689,7 @@
     <col min="7" max="7" style="4" width="15.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25" customFormat="1" s="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -697,7 +712,7 @@
         <v>6</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="73.5" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="87" customFormat="1" s="1">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
@@ -713,274 +728,334 @@
       <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="51" customFormat="1" s="1">
+      <c r="F2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="60" customFormat="1" s="1">
       <c r="A3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="51" customFormat="1" s="1">
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="60" customFormat="1" s="1">
       <c r="A4" s="3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="39.75" customFormat="1" s="1">
+        <v>23</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="46.5" customFormat="1" s="1">
       <c r="A5" s="3" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="73.5" customFormat="1" s="1">
+      <c r="A6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="60" customFormat="1" s="1">
+      <c r="A7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="73.5" customFormat="1" s="1">
+      <c r="A8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="60" customFormat="1" s="1">
+      <c r="A9" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="62.25" customFormat="1" s="1">
-      <c r="A6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="51" customFormat="1" s="1">
-      <c r="A7" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="62.25" customFormat="1" s="1">
-      <c r="A8" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="51" customFormat="1" s="1">
-      <c r="A9" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="51" customFormat="1" s="1">
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="60" customFormat="1" s="1">
       <c r="A10" s="3" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="51" customFormat="1" s="1">
+        <v>56</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="60" customFormat="1" s="1">
       <c r="A11" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="51" customFormat="1" s="1">
+        <v>61</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="60" customFormat="1" s="1">
       <c r="A12" s="3" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="51" customFormat="1" s="1">
+        <v>67</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="114" customFormat="1" s="1">
       <c r="A13" s="3" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
+        <v>72</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="51" customFormat="1" s="1">
       <c r="A14" s="3" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
+        <v>77</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="51" customFormat="1" s="1">
       <c r="A15" s="3" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
+        <v>83</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="51" customFormat="1" s="1">
       <c r="A16" s="3" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
+        <v>88</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>13</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>